<commit_message>
Task 2: BBT Testing - Updated repository, service tests
</commit_message>
<xml_diff>
--- a/Exam/gymtrackerpro/lib/repository/__tests__/bbt/exercise-repository/delete-bbt-form.xlsx
+++ b/Exam/gymtrackerpro/lib/repository/__tests__/bbt/exercise-repository/delete-bbt-form.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="80">
   <si>
     <t>Statement: ExerciseRepository.delete(id) – deletes exercise if not referenced in sessions.</t>
   </si>
@@ -142,31 +142,49 @@
     <t>ID length</t>
   </si>
   <si>
+    <t>id = "" (empty)</t>
+  </si>
+  <si>
+    <t>id = "a" (inexistent)</t>
+  </si>
+  <si>
+    <t>id = "a" (existing)</t>
+  </si>
+  <si>
+    <t>BVA</t>
+  </si>
+  <si>
+    <t>BVA-1 Zero</t>
+  </si>
+  <si>
+    <t>usageCount=0</t>
+  </si>
+  <si>
+    <t>BVA-2 One</t>
+  </si>
+  <si>
+    <t>usageCount=1</t>
+  </si>
+  <si>
+    <t>BVA-3 EmptyID</t>
+  </si>
+  <si>
     <t>id = ""</t>
   </si>
   <si>
-    <t>id = "a"</t>
-  </si>
-  <si>
-    <t>BVA</t>
-  </si>
-  <si>
-    <t>BVA-1 Zero</t>
-  </si>
-  <si>
-    <t>usageCount=0</t>
-  </si>
-  <si>
-    <t>BVA-2 One</t>
-  </si>
-  <si>
-    <t>usageCount=1</t>
-  </si>
-  <si>
-    <t>BVA-3 EmptyID</t>
-  </si>
-  <si>
-    <t>BVA-4 OneChar</t>
+    <t>BVA-4 InexChar</t>
+  </si>
+  <si>
+    <t>id = "a" (inex)</t>
+  </si>
+  <si>
+    <t>BVA-5 ExistChar</t>
+  </si>
+  <si>
+    <t>id = "a" (exist)</t>
+  </si>
+  <si>
+    <t>Resolves successfully</t>
   </si>
   <si>
     <t>TC from EC</t>
@@ -194,6 +212,9 @@
   </si>
   <si>
     <t>BVA-4</t>
+  </si>
+  <si>
+    <t>BVA-5</t>
   </si>
   <si>
     <t>Testing</t>
@@ -923,7 +944,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -986,6 +1007,17 @@
         <v>42</v>
       </c>
     </row>
+    <row r="6" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -994,7 +1026,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1009,7 +1041,7 @@
         <v>21</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>23</v>
@@ -1026,10 +1058,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>28</v>
@@ -1043,10 +1075,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>35</v>
@@ -1060,10 +1092,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>32</v>
@@ -1077,15 +1109,32 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E5" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1097,7 +1146,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1113,10 +1162,10 @@
         <v>21</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>23</v>
@@ -1139,7 +1188,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>28</v>
@@ -1159,7 +1208,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>32</v>
@@ -1179,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>35</v>
@@ -1196,10 +1245,10 @@
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>28</v>
@@ -1216,10 +1265,10 @@
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>35</v>
@@ -1236,10 +1285,10 @@
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>32</v>
@@ -1256,7 +1305,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>42</v>
@@ -1265,6 +1314,26 @@
         <v>32</v>
       </c>
       <c r="F8" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1293,16 +1362,16 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
@@ -1310,45 +1379,45 @@
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B3" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="1">
         <v>0</v>
@@ -1357,19 +1426,19 @@
         <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="H3" s="1">
         <v>0</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>